<commit_message>
family fantasy linked in
</commit_message>
<xml_diff>
--- a/data/leagues/2026 Family League 2026.xlsx
+++ b/data/leagues/2026 Family League 2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="94">
   <si>
     <t>Noah's Nifty Team</t>
   </si>
@@ -217,25 +217,22 @@
     <t>0-1</t>
   </si>
   <si>
-    <t>12.2-1.8-0.1</t>
-  </si>
-  <si>
-    <t>11.2-2.8-0.1</t>
-  </si>
-  <si>
-    <t>10.6-3.3-0.1</t>
+    <t>12.1-1.8-0.1</t>
+  </si>
+  <si>
+    <t>11.1-2.8-0.1</t>
+  </si>
+  <si>
+    <t>10.7-3.2-0.1</t>
   </si>
   <si>
     <t>10.2-3.7-0.1</t>
   </si>
   <si>
-    <t>8.0-5.9-0.1</t>
-  </si>
-  <si>
-    <t>6.0-7.8-0.1</t>
-  </si>
-  <si>
-    <t>6.0-7.9-0.1</t>
+    <t>8.0-6.0-0.1</t>
+  </si>
+  <si>
+    <t>6.1-7.8-0.1</t>
   </si>
   <si>
     <t>5.4-8.5-0.1</t>
@@ -244,25 +241,19 @@
     <t>4.4-9.5-0.1</t>
   </si>
   <si>
-    <t>4.1-9.8-0.1</t>
-  </si>
-  <si>
-    <t>3.2-10.7-0.1</t>
-  </si>
-  <si>
-    <t>2.2-11.7-0.1</t>
-  </si>
-  <si>
-    <t>13-1</t>
+    <t>3.9-10.0-0.1</t>
+  </si>
+  <si>
+    <t>3.3-10.7-0.1</t>
+  </si>
+  <si>
+    <t>2.3-11.7-0.1</t>
   </si>
   <si>
     <t>12-2</t>
   </si>
   <si>
     <t>11-3</t>
-  </si>
-  <si>
-    <t>10-4</t>
   </si>
   <si>
     <t>8-6</t>
@@ -1216,25 +1207,25 @@
   <sheetData>
     <row r="1" spans="2:8">
       <c r="B1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1713,22 +1704,22 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>62.7</v>
+        <v>61.4</v>
       </c>
       <c r="C2">
-        <v>25.1</v>
+        <v>22.4</v>
       </c>
       <c r="D2">
-        <v>8.4</v>
+        <v>12.1</v>
       </c>
       <c r="E2">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="F2">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1757,25 +1748,25 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="C3">
-        <v>34.7</v>
+        <v>34.2</v>
       </c>
       <c r="D3">
-        <v>26</v>
+        <v>25.4</v>
       </c>
       <c r="E3">
-        <v>14.5</v>
+        <v>16.7</v>
       </c>
       <c r="F3">
-        <v>3.7</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="H3">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1793,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1801,25 +1792,25 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>10.4</v>
+        <v>11.7</v>
       </c>
       <c r="C4">
-        <v>22.3</v>
+        <v>24.8</v>
       </c>
       <c r="D4">
-        <v>33.7</v>
+        <v>32.5</v>
       </c>
       <c r="E4">
-        <v>26.6</v>
+        <v>23.4</v>
       </c>
       <c r="F4">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
       <c r="G4">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H4">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1828,7 +1819,7 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -1837,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <v>99.5</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1845,34 +1836,34 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
       <c r="C5">
-        <v>16.6</v>
+        <v>17.8</v>
       </c>
       <c r="D5">
-        <v>27.1</v>
+        <v>26.2</v>
       </c>
       <c r="E5">
-        <v>36.7</v>
+        <v>38.8</v>
       </c>
       <c r="F5">
-        <v>10.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G5">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="H5">
         <v>0.5</v>
       </c>
       <c r="I5">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1881,7 +1872,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>99.3</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1889,43 +1880,43 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C6">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="D6">
-        <v>4.1</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
       <c r="F6">
-        <v>44</v>
+        <v>46.9</v>
       </c>
       <c r="G6">
-        <v>21.2</v>
+        <v>22.6</v>
       </c>
       <c r="H6">
-        <v>10.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I6">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="J6">
         <v>1.4</v>
       </c>
       <c r="K6">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="N6">
-        <v>84.09999999999999</v>
+        <v>86.09999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1933,43 +1924,43 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E7">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="F7">
-        <v>15.7</v>
+        <v>14.2</v>
       </c>
       <c r="G7">
-        <v>24.2</v>
+        <v>25.6</v>
       </c>
       <c r="H7">
-        <v>23.1</v>
+        <v>25</v>
       </c>
       <c r="I7">
-        <v>16.6</v>
+        <v>16</v>
       </c>
       <c r="J7">
-        <v>10.7</v>
+        <v>9.5</v>
       </c>
       <c r="K7">
-        <v>4.3</v>
+        <v>5.6</v>
       </c>
       <c r="L7">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="M7">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="N7">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1983,37 +1974,37 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E8">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="G8">
-        <v>27.2</v>
+        <v>26.3</v>
       </c>
       <c r="H8">
-        <v>22</v>
+        <v>22.8</v>
       </c>
       <c r="I8">
-        <v>17.3</v>
+        <v>16.8</v>
       </c>
       <c r="J8">
-        <v>11.5</v>
+        <v>10</v>
       </c>
       <c r="K8">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="L8">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="M8">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="N8">
-        <v>41.4</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -2027,37 +2018,37 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E9">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="G9">
-        <v>13.5</v>
+        <v>12.6</v>
       </c>
       <c r="H9">
-        <v>20.8</v>
+        <v>17.8</v>
       </c>
       <c r="I9">
-        <v>21.3</v>
+        <v>25.6</v>
       </c>
       <c r="J9">
-        <v>20.1</v>
+        <v>18.1</v>
       </c>
       <c r="K9">
-        <v>10.7</v>
+        <v>13.3</v>
       </c>
       <c r="L9">
-        <v>6.6</v>
+        <v>5.6</v>
       </c>
       <c r="M9">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="N9">
-        <v>19.6</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -2074,34 +2065,34 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F10">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="G10">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="H10">
-        <v>10.4</v>
+        <v>11.9</v>
       </c>
       <c r="I10">
-        <v>18.3</v>
+        <v>16.2</v>
       </c>
       <c r="J10">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="K10">
-        <v>19.2</v>
+        <v>20.1</v>
       </c>
       <c r="L10">
-        <v>15</v>
+        <v>13.9</v>
       </c>
       <c r="M10">
         <v>7.8</v>
       </c>
       <c r="N10">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -2112,40 +2103,40 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="G11">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="H11">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="I11">
-        <v>15.4</v>
+        <v>14</v>
       </c>
       <c r="J11">
-        <v>20.8</v>
+        <v>19.4</v>
       </c>
       <c r="K11">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="L11">
-        <v>17</v>
+        <v>19.9</v>
       </c>
       <c r="M11">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="N11">
-        <v>4.6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -2165,31 +2156,31 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="G12">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="H12">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="I12">
-        <v>6.4</v>
+        <v>7.3</v>
       </c>
       <c r="J12">
-        <v>9.800000000000001</v>
+        <v>13.3</v>
       </c>
       <c r="K12">
-        <v>22.3</v>
+        <v>17.7</v>
       </c>
       <c r="L12">
-        <v>32.6</v>
+        <v>33.1</v>
       </c>
       <c r="M12">
-        <v>24.1</v>
+        <v>23.3</v>
       </c>
       <c r="N12">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -2209,28 +2200,28 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="G13">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="H13">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I13">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="J13">
-        <v>3.3</v>
+        <v>5.5</v>
       </c>
       <c r="K13">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="L13">
-        <v>24.8</v>
+        <v>24</v>
       </c>
       <c r="M13">
-        <v>58.6</v>
+        <v>57.3</v>
       </c>
       <c r="N13">
         <v>0.4</v>
@@ -2256,7 +2247,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -2267,13 +2258,13 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>100</v>
       </c>
       <c r="C3">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2281,10 +2272,10 @@
         <v>6</v>
       </c>
       <c r="B4">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="C4">
         <v>99.8</v>
-      </c>
-      <c r="C4">
-        <v>99.7</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2292,10 +2283,10 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>99.59999999999999</v>
+        <v>99.8</v>
       </c>
       <c r="C5">
-        <v>99.3</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2303,10 +2294,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>87.40000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="C6">
-        <v>83.59999999999999</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2314,10 +2305,10 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>39.1</v>
+        <v>37.9</v>
       </c>
       <c r="C7">
-        <v>41.8</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2325,10 +2316,10 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>35.2</v>
+        <v>36.1</v>
       </c>
       <c r="C8">
-        <v>40.5</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2336,10 +2327,10 @@
         <v>4</v>
       </c>
       <c r="B9">
-        <v>23.1</v>
+        <v>23.9</v>
       </c>
       <c r="C9">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2347,10 +2338,10 @@
         <v>2</v>
       </c>
       <c r="B10">
-        <v>10.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C10">
-        <v>9.1</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2358,10 +2349,10 @@
         <v>5</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2369,10 +2360,10 @@
         <v>7</v>
       </c>
       <c r="B12">
-        <v>0.8999999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="C12">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2380,7 +2371,7 @@
         <v>3</v>
       </c>
       <c r="B13">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C13">
         <v>0.1</v>
@@ -2835,7 +2826,7 @@
         <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2855,7 +2846,7 @@
         <v>154.96</v>
       </c>
       <c r="F3">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2864,7 +2855,7 @@
         <v>65</v>
       </c>
       <c r="I3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2884,7 +2875,7 @@
         <v>152.3</v>
       </c>
       <c r="F4">
-        <v>99.5</v>
+        <v>99.8</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2893,7 +2884,7 @@
         <v>66</v>
       </c>
       <c r="I4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2913,7 +2904,7 @@
         <v>148.66</v>
       </c>
       <c r="F5">
-        <v>99.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2922,7 +2913,7 @@
         <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2942,16 +2933,16 @@
         <v>123.9</v>
       </c>
       <c r="F6">
-        <v>84.09999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H6" t="s">
         <v>68</v>
       </c>
       <c r="I6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2971,16 +2962,16 @@
         <v>119.96</v>
       </c>
       <c r="F7">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7">
-        <v>0.6</v>
+        <v>0.7000000000000001</v>
       </c>
       <c r="H7" t="s">
         <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -3000,16 +2991,16 @@
         <v>115.26</v>
       </c>
       <c r="F8">
-        <v>41.4</v>
+        <v>41.8</v>
       </c>
       <c r="G8">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="H8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -3029,16 +3020,16 @@
         <v>104.32</v>
       </c>
       <c r="F9">
-        <v>19.6</v>
+        <v>18.4</v>
       </c>
       <c r="G9">
-        <v>0.8999999999999999</v>
+        <v>1.2</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -3058,16 +3049,16 @@
         <v>100.32</v>
       </c>
       <c r="F10">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="G10">
         <v>7.8</v>
       </c>
       <c r="H10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -3087,16 +3078,16 @@
         <v>101.76</v>
       </c>
       <c r="F11">
-        <v>4.6</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3116,16 +3107,16 @@
         <v>92.06</v>
       </c>
       <c r="F12">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>24.1</v>
+        <v>23.3</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3148,13 +3139,13 @@
         <v>0.4</v>
       </c>
       <c r="G13">
-        <v>58.59999999999999</v>
+        <v>57.3</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -3172,16 +3163,16 @@
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3436,10 +3427,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:3">

</xml_diff>